<commit_message>
Convert euros through the P2P dollar, not the central bank rate
The owner's Excel prices the ruble by a single number, the P2P USDT rate,
and reaches euros via EUR/USD. A separate CBR euro rate would make every
row holding euros fail the import reconciliation.

The template generator now lives next to the template so the import
contract can be regenerated instead of hand-edited.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import/import-template.xlsx
+++ b/docs/import/import-template.xlsx
@@ -21,8 +21,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="#,##0&quot; ₽&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="#,##0&quot; ₽&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -109,9 +109,9 @@
     </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -581,7 +581,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   EUR/RUB — курс евро к рублю.</t>
+          <t xml:space="preserve">   EUR/USD — курс евро к доллару (ЕЦБ). Евро в рубли идёт через доллар: EUR/USD × USDT/RUB.</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   RUB × 1 · USD × USDT/RUB · EUR × EUR/RUB · BTC × BTC/USD × USDT/RUB</t>
+          <t xml:space="preserve">   RUB × 1 · USD × USDT/RUB · EUR × EUR/USD × USDT/RUB · BTC × BTC/USD × USDT/RUB</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>EUR/RUB</t>
+          <t>EUR/USD</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
@@ -1238,44 +1238,44 @@
       <c r="B4" s="11" t="n">
         <v>101</v>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>105</v>
-      </c>
-      <c r="D4" s="12" t="n">
+      <c r="C4" s="12" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="D4" s="13" t="n">
         <v>102000</v>
       </c>
-      <c r="E4" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F4:$AZ4*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B4+($F$2:$AZ$2="EUR")*$C4+($F$2:$AZ$2="BTC")*$D4*$B4)))</f>
-        <v/>
-      </c>
-      <c r="F4" s="12" t="n">
+      <c r="E4" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F4:$AZ4*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B4+($F$2:$AZ$2="EUR")*$C4*$B4+($F$2:$AZ$2="BTC")*$D4*$B4)))</f>
+        <v/>
+      </c>
+      <c r="F4" s="13" t="n">
         <v>420000</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="13" t="n">
         <v>85000</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="13" t="n">
         <v>3000</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="13" t="n">
         <v>50000</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="13" t="n">
         <v>1500</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="L4" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>0.25</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="N4" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O4" s="12" t="n">
+      <c r="O4" s="13" t="n">
         <v>240000</v>
       </c>
     </row>
@@ -1286,44 +1286,44 @@
       <c r="B5" s="11" t="n">
         <v>98.5</v>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>102</v>
-      </c>
-      <c r="D5" s="12" t="n">
+      <c r="C5" s="12" t="n">
+        <v>1.0355</v>
+      </c>
+      <c r="D5" s="13" t="n">
         <v>84000</v>
       </c>
-      <c r="E5" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F5:$AZ5*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B5+($F$2:$AZ$2="EUR")*$C5+($F$2:$AZ$2="BTC")*$D5*$B5)))</f>
-        <v/>
-      </c>
-      <c r="F5" s="12" t="n">
+      <c r="E5" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F5:$AZ5*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B5+($F$2:$AZ$2="EUR")*$C5*$B5+($F$2:$AZ$2="BTC")*$D5*$B5)))</f>
+        <v/>
+      </c>
+      <c r="F5" s="13" t="n">
         <v>450000</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="13" t="n">
         <v>90000</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="13" t="n">
         <v>3200</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="13" t="n">
         <v>40000</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="13" t="n">
         <v>45000</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="13" t="n">
         <v>1500</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="L5" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>0.26</v>
       </c>
-      <c r="N5" s="12" t="n">
+      <c r="N5" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O5" s="12" t="n">
+      <c r="O5" s="13" t="n">
         <v>210000</v>
       </c>
     </row>
@@ -1334,44 +1334,44 @@
       <c r="B6" s="11" t="n">
         <v>86</v>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>92</v>
-      </c>
-      <c r="D6" s="12" t="n">
+      <c r="C6" s="12" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="D6" s="13" t="n">
         <v>82500</v>
       </c>
-      <c r="E6" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F6:$AZ6*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B6+($F$2:$AZ$2="EUR")*$C6+($F$2:$AZ$2="BTC")*$D6*$B6)))</f>
-        <v/>
-      </c>
-      <c r="F6" s="12" t="n">
+      <c r="E6" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F6:$AZ6*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B6+($F$2:$AZ$2="EUR")*$C6*$B6+($F$2:$AZ$2="BTC")*$D6*$B6)))</f>
+        <v/>
+      </c>
+      <c r="F6" s="13" t="n">
         <v>380000</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="13" t="n">
         <v>70000</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="13" t="n">
         <v>3500</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="13" t="n">
         <v>60000</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="13" t="n">
         <v>400</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>0.275</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="N6" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O6" s="12" t="n">
+      <c r="O6" s="13" t="n">
         <v>180000</v>
       </c>
     </row>
@@ -1382,44 +1382,44 @@
       <c r="B7" s="11" t="n">
         <v>84</v>
       </c>
-      <c r="C7" s="11" t="n">
-        <v>94</v>
-      </c>
-      <c r="D7" s="12" t="n">
+      <c r="C7" s="12" t="n">
+        <v>1.135</v>
+      </c>
+      <c r="D7" s="13" t="n">
         <v>94000</v>
       </c>
-      <c r="E7" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F7:$AZ7*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B7+($F$2:$AZ$2="EUR")*$C7+($F$2:$AZ$2="BTC")*$D7*$B7)))</f>
-        <v/>
-      </c>
-      <c r="F7" s="12" t="n">
+      <c r="E7" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F7:$AZ7*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B7+($F$2:$AZ$2="EUR")*$C7*$B7+($F$2:$AZ$2="BTC")*$D7*$B7)))</f>
+        <v/>
+      </c>
+      <c r="F7" s="13" t="n">
         <v>410000</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <v>75000</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="13" t="n">
         <v>3500</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="13" t="n">
         <v>55000</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="13" t="n">
         <v>1800</v>
       </c>
-      <c r="L7" s="12" t="n">
+      <c r="L7" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="M7" s="12" t="n">
         <v>0.275</v>
       </c>
-      <c r="N7" s="12" t="n">
+      <c r="N7" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O7" s="12" t="n">
+      <c r="O7" s="13" t="n">
         <v>150000</v>
       </c>
     </row>
@@ -1430,44 +1430,44 @@
       <c r="B8" s="11" t="n">
         <v>80.5</v>
       </c>
-      <c r="C8" s="11" t="n">
-        <v>90</v>
-      </c>
-      <c r="D8" s="12" t="n">
+      <c r="C8" s="12" t="n">
+        <v>1.128</v>
+      </c>
+      <c r="D8" s="13" t="n">
         <v>104000</v>
       </c>
-      <c r="E8" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F8:$AZ8*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B8+($F$2:$AZ$2="EUR")*$C8+($F$2:$AZ$2="BTC")*$D8*$B8)))</f>
-        <v/>
-      </c>
-      <c r="F8" s="12" t="n">
+      <c r="E8" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F8:$AZ8*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B8+($F$2:$AZ$2="EUR")*$C8*$B8+($F$2:$AZ$2="BTC")*$D8*$B8)))</f>
+        <v/>
+      </c>
+      <c r="F8" s="13" t="n">
         <v>430000</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="13" t="n">
         <v>80000</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="13" t="n">
         <v>3600</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="12" t="n">
+      <c r="J8" s="13" t="n">
         <v>52000</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="L8" s="12" t="n">
+      <c r="L8" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="M8" s="14" t="n">
+      <c r="M8" s="12" t="n">
         <v>0.28</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O8" s="12" t="n">
+      <c r="O8" s="13" t="n">
         <v>120000</v>
       </c>
     </row>
@@ -1478,44 +1478,44 @@
       <c r="B9" s="11" t="n">
         <v>79</v>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>91</v>
-      </c>
-      <c r="D9" s="12" t="n">
+      <c r="C9" s="12" t="n">
+        <v>1.172</v>
+      </c>
+      <c r="D9" s="13" t="n">
         <v>107000</v>
       </c>
-      <c r="E9" s="13">
-        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F9:$AZ9*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B9+($F$2:$AZ$2="EUR")*$C9+($F$2:$AZ$2="BTC")*$D9*$B9)))</f>
-        <v/>
-      </c>
-      <c r="F9" s="12" t="n">
+      <c r="E9" s="14">
+        <f>IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F9:$AZ9*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B9+($F$2:$AZ$2="EUR")*$C9*$B9+($F$2:$AZ$2="BTC")*$D9*$B9)))</f>
+        <v/>
+      </c>
+      <c r="F9" s="13" t="n">
         <v>455000</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="13" t="n">
         <v>82000</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="13" t="n">
         <v>3600</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="13" t="n">
         <v>50000</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="13" t="n">
         <v>2000</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="13" t="n">
         <v>300</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>0.29</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="13" t="n">
         <v>1500000</v>
       </c>
-      <c r="O9" s="12" t="n">
+      <c r="O9" s="13" t="n">
         <v>90000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Warn in the template that Итог ₽ must be a pasted value, not the template formula
The template's total is a formula implementing the same rule as the app. If the
owner copies those rows down while building his sheet, the app reconciles against
itself and every transfer error shows "сошлось". The legend and the E3 comment now
say so explicitly. LAST_COL grows from AZ to DZ (~120 places, closed ones included).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/import/import-template.xlsx
+++ b/docs/import/import-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\quietfault\apps\networth-tracker\docs\import\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DADCB6F-01A6-4A26-9B71-09BC8D592865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47ADC02-C801-4878-889E-2CEC7EA18474}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13910" yWindow="6330" windowWidth="5630" windowHeight="4330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Как заполнять" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>В шаблоне — формула для образца. В вашем файле здесь итог, который считает ваш Excel: приложение сверит с ним свой.</t>
+          <t>В шаблоне здесь формула для образца. В вашем файле нужно число из вашей главной вкладки (значения или ссылка на её итог), а не эта формула: иначе приложение сверит само себя.</t>
         </r>
       </text>
     </comment>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="54">
   <si>
     <t>Шаблон импорта истории в «Срез»</t>
   </si>
@@ -101,7 +101,10 @@
     <t xml:space="preserve">   Итог ₽ — итог по вашему Excel. Приложение посчитает свой и покажет строки, где они разошлись.</t>
   </si>
   <si>
-    <t xml:space="preserve">   Дальше — колонки мест, сколько угодно, в валюте места. Новое место — новая колонка справа</t>
+    <t>В «Итог ₽» — число из вашей главной вкладки (Специальная вставка → Значения) или ссылка на её итог. Формулу шаблона не оставляйте: иначе приложение сверит само себя и любая ошибка переноса покажет «сошлось».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Дальше — колонки мест (до ~120, закрытые тоже считаются), в валюте места. Новое место — новая колонка справа</t>
   </si>
   <si>
     <t xml:space="preserve">   плюс строка на листе «Места». Место закрылось — ставьте 0, колонку не удаляйте.</t>
@@ -624,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
@@ -701,7 +704,7 @@
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
     </row>
@@ -710,8 +713,8 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A20" s="4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -720,19 +723,24 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" s="3" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" s="4" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" s="4" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -752,156 +760,156 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -919,7 +927,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AZ9"/>
+  <dimension ref="A1:DZ9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -928,14 +936,14 @@
     <col min="6" max="15" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:130" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="2" spans="1:130" x14ac:dyDescent="0.35">
       <c r="E2" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="8" t="str">
         <f>IF(F$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(F$3,Места!$A:$A,0)),"?"))</f>
@@ -1125,55 +1133,367 @@
         <f>IF(AZ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(AZ$3,Места!$A:$A,0)),"?"))</f>
         <v/>
       </c>
-    </row>
-    <row r="3" spans="1:52" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="BA2" s="8" t="str">
+        <f>IF(BA$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BA$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BB2" s="8" t="str">
+        <f>IF(BB$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BB$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BC2" s="8" t="str">
+        <f>IF(BC$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BC$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BD2" s="8" t="str">
+        <f>IF(BD$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BD$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BE2" s="8" t="str">
+        <f>IF(BE$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BE$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BF2" s="8" t="str">
+        <f>IF(BF$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BF$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BG2" s="8" t="str">
+        <f>IF(BG$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BG$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BH2" s="8" t="str">
+        <f>IF(BH$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BH$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BI2" s="8" t="str">
+        <f>IF(BI$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BI$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BJ2" s="8" t="str">
+        <f>IF(BJ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BJ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BK2" s="8" t="str">
+        <f>IF(BK$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BK$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BL2" s="8" t="str">
+        <f>IF(BL$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BL$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BM2" s="8" t="str">
+        <f>IF(BM$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BM$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BN2" s="8" t="str">
+        <f>IF(BN$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BN$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BO2" s="8" t="str">
+        <f>IF(BO$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BO$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BP2" s="8" t="str">
+        <f>IF(BP$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BP$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BQ2" s="8" t="str">
+        <f>IF(BQ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BQ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BR2" s="8" t="str">
+        <f>IF(BR$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BR$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BS2" s="8" t="str">
+        <f>IF(BS$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BS$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BT2" s="8" t="str">
+        <f>IF(BT$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BT$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BU2" s="8" t="str">
+        <f>IF(BU$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BU$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BV2" s="8" t="str">
+        <f>IF(BV$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BV$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BW2" s="8" t="str">
+        <f>IF(BW$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BW$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BX2" s="8" t="str">
+        <f>IF(BX$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BX$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BY2" s="8" t="str">
+        <f>IF(BY$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BY$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="BZ2" s="8" t="str">
+        <f>IF(BZ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(BZ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CA2" s="8" t="str">
+        <f>IF(CA$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CA$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CB2" s="8" t="str">
+        <f>IF(CB$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CB$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CC2" s="8" t="str">
+        <f>IF(CC$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CC$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CD2" s="8" t="str">
+        <f>IF(CD$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CD$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CE2" s="8" t="str">
+        <f>IF(CE$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CE$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CF2" s="8" t="str">
+        <f>IF(CF$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CF$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CG2" s="8" t="str">
+        <f>IF(CG$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CG$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CH2" s="8" t="str">
+        <f>IF(CH$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CH$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CI2" s="8" t="str">
+        <f>IF(CI$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CI$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CJ2" s="8" t="str">
+        <f>IF(CJ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CJ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CK2" s="8" t="str">
+        <f>IF(CK$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CK$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CL2" s="8" t="str">
+        <f>IF(CL$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CL$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CM2" s="8" t="str">
+        <f>IF(CM$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CM$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CN2" s="8" t="str">
+        <f>IF(CN$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CN$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CO2" s="8" t="str">
+        <f>IF(CO$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CO$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CP2" s="8" t="str">
+        <f>IF(CP$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CP$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CQ2" s="8" t="str">
+        <f>IF(CQ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CQ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CR2" s="8" t="str">
+        <f>IF(CR$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CR$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CS2" s="8" t="str">
+        <f>IF(CS$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CS$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CT2" s="8" t="str">
+        <f>IF(CT$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CT$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CU2" s="8" t="str">
+        <f>IF(CU$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CU$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CV2" s="8" t="str">
+        <f>IF(CV$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CV$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CW2" s="8" t="str">
+        <f>IF(CW$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CW$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CX2" s="8" t="str">
+        <f>IF(CX$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CX$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CY2" s="8" t="str">
+        <f>IF(CY$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CY$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="CZ2" s="8" t="str">
+        <f>IF(CZ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(CZ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DA2" s="8" t="str">
+        <f>IF(DA$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DA$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DB2" s="8" t="str">
+        <f>IF(DB$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DB$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DC2" s="8" t="str">
+        <f>IF(DC$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DC$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DD2" s="8" t="str">
+        <f>IF(DD$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DD$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DE2" s="8" t="str">
+        <f>IF(DE$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DE$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DF2" s="8" t="str">
+        <f>IF(DF$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DF$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DG2" s="8" t="str">
+        <f>IF(DG$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DG$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DH2" s="8" t="str">
+        <f>IF(DH$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DH$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DI2" s="8" t="str">
+        <f>IF(DI$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DI$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DJ2" s="8" t="str">
+        <f>IF(DJ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DJ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DK2" s="8" t="str">
+        <f>IF(DK$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DK$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DL2" s="8" t="str">
+        <f>IF(DL$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DL$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DM2" s="8" t="str">
+        <f>IF(DM$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DM$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DN2" s="8" t="str">
+        <f>IF(DN$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DN$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DO2" s="8" t="str">
+        <f>IF(DO$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DO$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DP2" s="8" t="str">
+        <f>IF(DP$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DP$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DQ2" s="8" t="str">
+        <f>IF(DQ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DQ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DR2" s="8" t="str">
+        <f>IF(DR$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DR$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DS2" s="8" t="str">
+        <f>IF(DS$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DS$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DT2" s="8" t="str">
+        <f>IF(DT$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DT$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DU2" s="8" t="str">
+        <f>IF(DU$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DU$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DV2" s="8" t="str">
+        <f>IF(DV$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DV$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DW2" s="8" t="str">
+        <f>IF(DW$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DW$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DX2" s="8" t="str">
+        <f>IF(DX$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DX$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DY2" s="8" t="str">
+        <f>IF(DY$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DY$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+      <c r="DZ2" s="8" t="str">
+        <f>IF(DZ$3="","",IFERROR(INDEX(Места!$C:$C,MATCH(DZ$3,Места!$A:$A,0)),"?"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:130" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A4" s="10">
         <v>45688</v>
       </c>
@@ -1187,7 +1507,7 @@
         <v>102000</v>
       </c>
       <c r="E4" s="14">
-        <f t="shared" ref="E4:E9" si="0">IF(COUNTIF($F$2:$AZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F4:$AZ4*(($F$2:$AZ$2="RUB")+($F$2:$AZ$2="USD")*$B4+($F$2:$AZ$2="EUR")*$C4*$B4+($F$2:$AZ$2="BTC")*$D4*$B4)))</f>
+        <f t="shared" ref="E4:E9" si="0">IF(COUNTIF($F$2:$DZ$2,"?")&gt;0,"нет в «Места»",SUMPRODUCT($F4:$DZ4*(($F$2:$DZ$2="RUB")+($F$2:$DZ$2="USD")*$B4+($F$2:$DZ$2="EUR")*$C4*$B4+($F$2:$DZ$2="BTC")*$D4*$B4)))</f>
         <v>5427016</v>
       </c>
       <c r="F4" s="13">
@@ -1221,7 +1541,7 @@
         <v>240000</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A5" s="10">
         <v>45716</v>
       </c>
@@ -1269,7 +1589,7 @@
         <v>210000</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A6" s="10">
         <v>45747</v>
       </c>
@@ -1317,7 +1637,7 @@
         <v>180000</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
         <v>45777</v>
       </c>
@@ -1365,7 +1685,7 @@
         <v>150000</v>
       </c>
     </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>45808</v>
       </c>
@@ -1413,7 +1733,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:130" x14ac:dyDescent="0.35">
       <c r="A9" s="10">
         <v>45838</v>
       </c>

</xml_diff>